<commit_message>
Markowitz and Efficiency Curve
</commit_message>
<xml_diff>
--- a/Open Positions.xlsx
+++ b/Open Positions.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Professional_WorkTools\Github\RodWal-Portfolio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Professional_WorkTools\Github\StockSillines\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C550248E-F68A-456F-B0DD-568EDE7F7AA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{879A82F2-D606-405C-815B-A5C5FB79C475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Positions" sheetId="1" r:id="rId1"/>
@@ -45,9 +45,6 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Ticket</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
@@ -298,6 +295,9 @@
   </si>
   <si>
     <t>Risk Mix</t>
+  </si>
+  <si>
+    <t>Ticker</t>
   </si>
 </sst>
 </file>
@@ -706,16 +706,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:S32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.42578125" style="8" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="9.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9" style="1" customWidth="1"/>
     <col min="8" max="8" width="9.85546875" style="10" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.42578125" style="10" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.140625" style="10"/>
@@ -732,72 +733,72 @@
   <sheetData>
     <row r="1" spans="1:19" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B1" s="16" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="E1" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="F1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="G1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="19" t="s">
-        <v>5</v>
-      </c>
       <c r="H1" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="I1" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="K1" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L1" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M1" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="N1" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="I1" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="K1" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="L1" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="M1" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="N1" s="16" t="s">
+      <c r="O1" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="O1" s="16" t="s">
+      <c r="P1" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="Q1" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="Q1" s="16" t="s">
+      <c r="R1" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="S1" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="R1" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="S1" s="16" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D2" s="8">
         <v>45507</v>
@@ -806,27 +807,33 @@
         <v>9.9999999999999998E-46</v>
       </c>
       <c r="F2" s="1">
-        <v>63.3</v>
+        <v>41.8</v>
       </c>
       <c r="G2" s="1">
         <f t="shared" ref="G2:G31" si="0">E2*F2</f>
-        <v>6.3299999999999997E-44</v>
-      </c>
-      <c r="J2" s="9" t="str">
+        <v>4.1799999999999994E-44</v>
+      </c>
+      <c r="H2" s="11">
+        <v>0</v>
+      </c>
+      <c r="I2" s="11">
+        <v>0.4</v>
+      </c>
+      <c r="J2" s="9">
         <f t="shared" ref="J2:J31" si="1">IFERROR(H2/I2,"")</f>
-        <v/>
-      </c>
-      <c r="K2" s="9" t="str">
+        <v>0</v>
+      </c>
+      <c r="K2" s="9">
         <f t="shared" ref="K2:K32" si="2">IFERROR(J2/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L2" s="12">
         <f t="shared" ref="L2:L31" si="3">F2/(1-(F2*(1+H2)-F2)/(F2*(1+H2)))</f>
-        <v>63.3</v>
+        <v>41.8</v>
       </c>
       <c r="M2" s="12">
         <f t="shared" ref="M2:M31" si="4">F2/(1+I2-H2)</f>
-        <v>63.3</v>
+        <v>29.857142857142858</v>
       </c>
       <c r="N2" s="12">
         <f t="shared" ref="N2:N31" si="5">L2-F2</f>
@@ -834,34 +841,34 @@
       </c>
       <c r="O2" s="12">
         <f t="shared" ref="O2:O31" si="6">0.5*(M2-F2)</f>
-        <v>0</v>
+        <v>-5.9714285714285698</v>
       </c>
       <c r="P2" s="15">
         <f t="shared" ref="P2:P31" si="7">N2+O2</f>
-        <v>0</v>
+        <v>-5.9714285714285698</v>
       </c>
       <c r="Q2" s="12">
         <f>MAX($P$2:$P$280)-P2</f>
-        <v>38.33801960784308</v>
+        <v>89.398549926326339</v>
       </c>
       <c r="R2" s="9">
         <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q2)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
-        <v>2.6083767764452363E-2</v>
+        <v>1.1185863762042041E-2</v>
       </c>
       <c r="S2" s="9">
         <f t="shared" ref="S2:S32" si="8">Q2/MAX($Q$2:$Q$28)</f>
-        <v>0.88019658171881077</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0.29521259291506552</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D3" s="8">
         <v>45574</v>
@@ -870,62 +877,69 @@
         <v>9.9999999999999998E-46</v>
       </c>
       <c r="F3" s="1">
-        <v>46.53</v>
+        <v>47.42</v>
       </c>
       <c r="G3" s="1">
         <f t="shared" si="0"/>
-        <v>4.6529999999999999E-44</v>
-      </c>
-      <c r="J3" s="9" t="str">
+        <v>4.7420000000000006E-44</v>
+      </c>
+      <c r="H3" s="11">
+        <f>48.37/F3-1</f>
+        <v>2.0033741037536856E-2</v>
+      </c>
+      <c r="I3" s="11">
+        <v>0.4</v>
+      </c>
+      <c r="J3" s="9">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K3" s="9" t="str">
+        <v>5.0084352593842141E-2</v>
+      </c>
+      <c r="K3" s="9">
         <f t="shared" si="2"/>
-        <v/>
+        <v>1.0095425032941828E-2</v>
       </c>
       <c r="L3" s="12">
         <f t="shared" si="3"/>
-        <v>46.53</v>
+        <v>48.37</v>
       </c>
       <c r="M3" s="12">
         <f t="shared" si="4"/>
-        <v>46.53</v>
+        <v>34.36315902075247</v>
       </c>
       <c r="N3" s="12">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.94999999999999574</v>
       </c>
       <c r="O3" s="12">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-6.5284204896237661</v>
       </c>
       <c r="P3" s="15">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>-5.5784204896237704</v>
       </c>
       <c r="Q3" s="12">
         <f t="shared" ref="Q3:Q32" si="9">MAX($P$2:$P$280)-P3</f>
-        <v>38.33801960784308</v>
+        <v>89.005541844521531</v>
       </c>
       <c r="R3" s="9">
         <f t="shared" ref="R3:R32" si="10">IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q3)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
-        <v>2.6083767764452363E-2</v>
+        <v>1.1235255460236852E-2</v>
       </c>
       <c r="S3" s="9">
         <f t="shared" si="8"/>
-        <v>0.88019658171881077</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0.29391479854410774</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="14" t="s">
         <v>32</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>33</v>
       </c>
       <c r="D4" s="8">
         <v>45511</v>
@@ -940,6 +954,8 @@
         <f t="shared" si="0"/>
         <v>1.1348000000000001E-20</v>
       </c>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
       <c r="J4" s="9" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -970,26 +986,26 @@
       </c>
       <c r="Q4" s="12">
         <f t="shared" si="9"/>
-        <v>38.33801960784308</v>
+        <v>83.427121354897764</v>
       </c>
       <c r="R4" s="9">
         <f t="shared" si="10"/>
-        <v>2.6083767764452363E-2</v>
+        <v>1.1986509707628705E-2</v>
       </c>
       <c r="S4" s="9">
         <f t="shared" si="8"/>
-        <v>0.88019658171881077</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0.27549369463951967</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D5" s="8">
         <v>45511</v>
@@ -1004,6 +1020,8 @@
         <f t="shared" si="0"/>
         <v>1.5740000000000001E-21</v>
       </c>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
       <c r="J5" s="9" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1034,26 +1052,26 @@
       </c>
       <c r="Q5" s="12">
         <f t="shared" si="9"/>
-        <v>38.33801960784308</v>
+        <v>83.427121354897764</v>
       </c>
       <c r="R5" s="9">
         <f t="shared" si="10"/>
-        <v>2.6083767764452363E-2</v>
+        <v>1.1986509707628705E-2</v>
       </c>
       <c r="S5" s="9">
         <f t="shared" si="8"/>
-        <v>0.88019658171881077</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0.27549369463951967</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D6" s="8">
         <v>45511</v>
@@ -1068,6 +1086,8 @@
         <f t="shared" si="0"/>
         <v>2.3091E-20</v>
       </c>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
       <c r="J6" s="9" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1098,26 +1118,26 @@
       </c>
       <c r="Q6" s="12">
         <f t="shared" si="9"/>
-        <v>38.33801960784308</v>
+        <v>83.427121354897764</v>
       </c>
       <c r="R6" s="9">
         <f t="shared" si="10"/>
-        <v>2.6083767764452363E-2</v>
+        <v>1.1986509707628705E-2</v>
       </c>
       <c r="S6" s="9">
         <f t="shared" si="8"/>
-        <v>0.88019658171881077</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0.27549369463951967</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D7" s="8">
         <v>45511</v>
@@ -1132,6 +1152,8 @@
         <f t="shared" si="0"/>
         <v>2.0110000000000001E-21</v>
       </c>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
       <c r="J7" s="9" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1162,26 +1184,26 @@
       </c>
       <c r="Q7" s="12">
         <f t="shared" si="9"/>
-        <v>38.33801960784308</v>
+        <v>83.427121354897764</v>
       </c>
       <c r="R7" s="9">
         <f t="shared" si="10"/>
-        <v>2.6083767764452363E-2</v>
+        <v>1.1986509707628705E-2</v>
       </c>
       <c r="S7" s="9">
         <f t="shared" si="8"/>
-        <v>0.88019658171881077</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0.27549369463951967</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B8" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" t="s">
         <v>55</v>
-      </c>
-      <c r="C8" t="s">
-        <v>56</v>
       </c>
       <c r="D8" s="8">
         <v>45511</v>
@@ -1196,6 +1218,8 @@
         <f t="shared" si="0"/>
         <v>1.2800000000000001E-21</v>
       </c>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
       <c r="J8" s="9" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1226,516 +1250,518 @@
       </c>
       <c r="Q8" s="12">
         <f t="shared" si="9"/>
-        <v>38.33801960784308</v>
+        <v>83.427121354897764</v>
       </c>
       <c r="R8" s="9">
         <f t="shared" si="10"/>
-        <v>2.6083767764452363E-2</v>
+        <v>1.1986509707628705E-2</v>
       </c>
       <c r="S8" s="9">
         <f t="shared" si="8"/>
-        <v>0.88019658171881077</v>
+        <v>0.27549369463951967</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>8</v>
+        <v>36</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="D9" s="8">
-        <v>45511</v>
+        <v>45574</v>
       </c>
       <c r="E9" s="2">
-        <v>0.14610000000000001</v>
+        <v>0.13370000000000001</v>
       </c>
       <c r="F9" s="1">
-        <v>273.45999999999998</v>
+        <v>423.77</v>
       </c>
       <c r="G9" s="1">
-        <f t="shared" si="0"/>
-        <v>39.952506</v>
+        <f>E9*F9</f>
+        <v>56.658049000000005</v>
       </c>
       <c r="H9" s="11">
-        <v>0.15</v>
+        <v>1.14E-2</v>
       </c>
       <c r="I9" s="11">
-        <v>0.17</v>
+        <v>0.1963</v>
       </c>
       <c r="J9" s="9">
-        <f t="shared" si="1"/>
-        <v>0.88235294117647045</v>
+        <f>IFERROR(H9/I9,"")</f>
+        <v>5.8074375955170655E-2</v>
       </c>
       <c r="K9" s="9">
-        <f t="shared" si="2"/>
-        <v>9.6518568995655959E-2</v>
+        <f>IFERROR(J9/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>1.1705961611299503E-2</v>
       </c>
       <c r="L9" s="12">
-        <f t="shared" si="3"/>
-        <v>314.47899999999993</v>
+        <f>F9/(1-(F9*(1+H9)-F9)/(F9*(1+H9)))</f>
+        <v>428.600978</v>
       </c>
       <c r="M9" s="12">
-        <f t="shared" si="4"/>
-        <v>268.09803921568624</v>
+        <f>F9/(1+I9-H9)</f>
+        <v>357.64199510507217</v>
       </c>
       <c r="N9" s="12">
-        <f t="shared" si="5"/>
-        <v>41.018999999999949</v>
+        <f>L9-F9</f>
+        <v>4.830978000000016</v>
       </c>
       <c r="O9" s="12">
-        <f t="shared" si="6"/>
-        <v>-2.6809803921568687</v>
+        <f>0.5*(M9-F9)</f>
+        <v>-33.064002447463906</v>
       </c>
       <c r="P9" s="15">
-        <f t="shared" si="7"/>
-        <v>38.33801960784308</v>
+        <f>N9+O9</f>
+        <v>-28.23302444746389</v>
       </c>
       <c r="Q9" s="12">
-        <f t="shared" si="9"/>
-        <v>0</v>
+        <f>MAX($P$2:$P$280)-P9</f>
+        <v>111.66014580236165</v>
       </c>
       <c r="R9" s="9">
-        <f t="shared" si="10"/>
-        <v>0</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q9)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>8.9557468585971488E-3</v>
       </c>
       <c r="S9" s="9">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <f>Q9/MAX($Q$2:$Q$28)</f>
+        <v>0.36872500946329412</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>43</v>
+        <v>38</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="D10" s="8">
-        <v>45580</v>
+        <v>45553</v>
       </c>
       <c r="E10" s="2">
-        <v>0.19139999999999999</v>
+        <v>1.0751999999999999</v>
       </c>
       <c r="F10" s="1">
-        <v>135.82</v>
+        <v>51.15</v>
       </c>
       <c r="G10" s="1">
-        <f t="shared" si="0"/>
-        <v>25.995947999999999</v>
+        <f>E10*F10</f>
+        <v>54.996479999999998</v>
       </c>
       <c r="H10" s="11">
-        <v>0.15</v>
+        <f>16.68%+7%/4</f>
+        <v>0.18430000000000002</v>
       </c>
       <c r="I10" s="11">
-        <v>0.22</v>
+        <v>0.19980000000000001</v>
       </c>
       <c r="J10" s="9">
-        <f t="shared" si="1"/>
-        <v>0.68181818181818177</v>
+        <f>IFERROR(H10/I10,"")</f>
+        <v>0.92242242242242245</v>
       </c>
       <c r="K10" s="9">
-        <f t="shared" si="2"/>
-        <v>7.4582530587552348E-2</v>
+        <f>IFERROR(J10/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>0.18593125261671253</v>
       </c>
       <c r="L10" s="12">
-        <f t="shared" si="3"/>
-        <v>156.19299999999998</v>
+        <f>F10/(1-(F10*(1+H10)-F10)/(F10*(1+H10)))</f>
+        <v>60.576944999999995</v>
       </c>
       <c r="M10" s="12">
-        <f t="shared" si="4"/>
-        <v>126.93457943925232</v>
+        <f>F10/(1+I10-H10)</f>
+        <v>50.369276218611525</v>
       </c>
       <c r="N10" s="12">
-        <f t="shared" si="5"/>
-        <v>20.37299999999999</v>
+        <f>L10-F10</f>
+        <v>9.4269449999999964</v>
       </c>
       <c r="O10" s="12">
-        <f t="shared" si="6"/>
-        <v>-4.4427102803738379</v>
+        <f>0.5*(M10-F10)</f>
+        <v>-0.39036189069423699</v>
       </c>
       <c r="P10" s="15">
-        <f t="shared" si="7"/>
-        <v>15.930289719626153</v>
+        <f>N10+O10</f>
+        <v>9.0365831093057594</v>
       </c>
       <c r="Q10" s="12">
-        <f t="shared" si="9"/>
-        <v>22.407729888216927</v>
+        <f>MAX($P$2:$P$280)-P10</f>
+        <v>74.390538245592012</v>
       </c>
       <c r="R10" s="9">
-        <f t="shared" si="10"/>
-        <v>4.4627456908334501E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q10)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.3442569762012102E-2</v>
       </c>
       <c r="S10" s="9">
-        <f t="shared" si="8"/>
-        <v>0.51445555752316563</v>
+        <f>Q10/MAX($Q$2:$Q$28)</f>
+        <v>0.24565301900228498</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>27</v>
+        <v>36</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="D11" s="8">
-        <v>45511</v>
+        <v>45482</v>
       </c>
       <c r="E11" s="2">
-        <v>0.1933</v>
+        <v>0.18820000000000001</v>
       </c>
       <c r="F11" s="1">
-        <v>77.53</v>
+        <v>227.38</v>
       </c>
       <c r="G11" s="1">
-        <f t="shared" si="0"/>
-        <v>14.986549</v>
+        <f>E11*F11</f>
+        <v>42.792915999999998</v>
       </c>
       <c r="H11" s="11">
-        <v>0.15</v>
+        <v>4.9299999999999997E-2</v>
       </c>
       <c r="I11" s="11">
-        <v>0.26</v>
+        <v>0.2271</v>
       </c>
       <c r="J11" s="9">
-        <f t="shared" si="1"/>
-        <v>0.57692307692307687</v>
+        <f>IFERROR(H11/I11,"")</f>
+        <v>0.21708498458828709</v>
       </c>
       <c r="K11" s="9">
-        <f t="shared" si="2"/>
-        <v>6.3108295112544288E-2</v>
+        <f>IFERROR(J11/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>4.3757482610603554E-2</v>
       </c>
       <c r="L11" s="12">
-        <f t="shared" si="3"/>
-        <v>89.159499999999994</v>
+        <f>F11/(1-(F11*(1+H11)-F11)/(F11*(1+H11)))</f>
+        <v>238.58983399999997</v>
       </c>
       <c r="M11" s="12">
-        <f t="shared" si="4"/>
-        <v>69.846846846846844</v>
+        <f>F11/(1+I11-H11)</f>
+        <v>193.05484802173541</v>
       </c>
       <c r="N11" s="12">
-        <f t="shared" si="5"/>
-        <v>11.629499999999993</v>
+        <f>L11-F11</f>
+        <v>11.209833999999972</v>
       </c>
       <c r="O11" s="12">
-        <f t="shared" si="6"/>
-        <v>-3.8415765765765784</v>
+        <f>0.5*(M11-F11)</f>
+        <v>-17.162575989132293</v>
       </c>
       <c r="P11" s="15">
-        <f t="shared" si="7"/>
-        <v>7.7879234234234147</v>
+        <f>N11+O11</f>
+        <v>-5.9527419891323206</v>
       </c>
       <c r="Q11" s="12">
-        <f t="shared" si="9"/>
-        <v>30.550096184419665</v>
+        <f>MAX($P$2:$P$280)-P11</f>
+        <v>89.379863344030085</v>
       </c>
       <c r="R11" s="9">
-        <f t="shared" si="10"/>
-        <v>3.2733121164770444E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q11)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.1188202382352297E-2</v>
       </c>
       <c r="S11" s="9">
-        <f t="shared" si="8"/>
-        <v>0.70139486879510005</v>
+        <f>Q11/MAX($Q$2:$Q$28)</f>
+        <v>0.29515088593640709</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>24</v>
+      <c r="B12" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="C12" t="s">
         <v>25</v>
       </c>
       <c r="D12" s="8">
-        <v>45482</v>
+        <v>45511</v>
       </c>
       <c r="E12" s="2">
-        <v>0.15210000000000001</v>
+        <v>0.14610000000000001</v>
       </c>
       <c r="F12" s="1">
-        <v>131.38</v>
+        <v>273.45999999999998</v>
       </c>
       <c r="G12" s="1">
-        <f t="shared" si="0"/>
-        <v>19.982898000000002</v>
+        <f>E12*F12</f>
+        <v>39.952506</v>
       </c>
       <c r="H12" s="11">
-        <v>0.3</v>
+        <v>0.16769999999999999</v>
       </c>
       <c r="I12" s="11">
-        <v>0.52</v>
+        <v>0.16700000000000001</v>
       </c>
       <c r="J12" s="9">
-        <f t="shared" si="1"/>
-        <v>0.57692307692307687</v>
+        <f>IFERROR(H12/I12,"")</f>
+        <v>1.0041916167664668</v>
       </c>
       <c r="K12" s="9">
-        <f t="shared" si="2"/>
-        <v>6.3108295112544288E-2</v>
+        <f>IFERROR(J12/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>0.20241334190712787</v>
       </c>
       <c r="L12" s="12">
-        <f t="shared" si="3"/>
-        <v>170.79400000000001</v>
+        <f>F12/(1-(F12*(1+H12)-F12)/(F12*(1+H12)))</f>
+        <v>319.31924199999997</v>
       </c>
       <c r="M12" s="12">
-        <f t="shared" si="4"/>
-        <v>107.68852459016394</v>
+        <f>F12/(1+I12-H12)</f>
+        <v>273.65155608926244</v>
       </c>
       <c r="N12" s="12">
-        <f t="shared" si="5"/>
-        <v>39.414000000000016</v>
+        <f>L12-F12</f>
+        <v>45.859241999999995</v>
       </c>
       <c r="O12" s="12">
-        <f t="shared" si="6"/>
-        <v>-11.845737704918029</v>
+        <f>0.5*(M12-F12)</f>
+        <v>9.5778044631231296E-2</v>
       </c>
       <c r="P12" s="15">
-        <f t="shared" si="7"/>
-        <v>27.568262295081986</v>
+        <f>N12+O12</f>
+        <v>45.955020044631226</v>
       </c>
       <c r="Q12" s="12">
-        <f t="shared" si="9"/>
-        <v>10.769757312761094</v>
+        <f>MAX($P$2:$P$280)-P12</f>
+        <v>37.472101310266538</v>
       </c>
       <c r="R12" s="9">
-        <f t="shared" si="10"/>
-        <v>9.2852602984386592E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q12)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>2.6686520505483952E-2</v>
       </c>
       <c r="S12" s="9">
-        <f t="shared" si="8"/>
-        <v>0.24726116971086817</v>
+        <f>Q12/MAX($Q$2:$Q$28)</f>
+        <v>0.12374066692240798</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="D13" s="8">
-        <v>45484</v>
+        <v>45544</v>
       </c>
       <c r="E13" s="2">
-        <v>0.18179999999999999</v>
+        <v>0.1928</v>
       </c>
       <c r="F13" s="1">
-        <v>192.37</v>
+        <v>188.12</v>
       </c>
       <c r="G13" s="1">
-        <f t="shared" si="0"/>
-        <v>34.972865999999996</v>
+        <f>E13*F13</f>
+        <v>36.269536000000002</v>
       </c>
       <c r="H13" s="11">
-        <v>0.2</v>
+        <v>-6.8599999999999994E-2</v>
       </c>
       <c r="I13" s="11">
-        <v>0.35</v>
+        <v>0.37780000000000002</v>
       </c>
       <c r="J13" s="9">
-        <f t="shared" si="1"/>
-        <v>0.57142857142857151</v>
+        <f>IFERROR(H13/I13,"")</f>
+        <v>-0.18157755426151401</v>
       </c>
       <c r="K13" s="9">
-        <f t="shared" si="2"/>
-        <v>6.2507263730520068E-2</v>
+        <f>IFERROR(J13/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>-3.6600305120793777E-2</v>
       </c>
       <c r="L13" s="12">
-        <f t="shared" si="3"/>
-        <v>230.84399999999999</v>
+        <f>F13/(1-(F13*(1+H13)-F13)/(F13*(1+H13)))</f>
+        <v>175.214968</v>
       </c>
       <c r="M13" s="12">
-        <f t="shared" si="4"/>
-        <v>167.2782608695652</v>
+        <f>F13/(1+I13-H13)</f>
+        <v>130.06084070796459</v>
       </c>
       <c r="N13" s="12">
-        <f t="shared" si="5"/>
-        <v>38.47399999999999</v>
+        <f>L13-F13</f>
+        <v>-12.905032000000006</v>
       </c>
       <c r="O13" s="12">
-        <f t="shared" si="6"/>
-        <v>-12.545869565217401</v>
+        <f>0.5*(M13-F13)</f>
+        <v>-29.029579646017709</v>
       </c>
       <c r="P13" s="15">
-        <f t="shared" si="7"/>
-        <v>25.928130434782588</v>
+        <f>N13+O13</f>
+        <v>-41.934611646017714</v>
       </c>
       <c r="Q13" s="12">
-        <f t="shared" si="9"/>
-        <v>12.409889173060492</v>
+        <f>MAX($P$2:$P$280)-P13</f>
+        <v>125.36173300091548</v>
       </c>
       <c r="R13" s="9">
-        <f t="shared" si="10"/>
-        <v>8.058089690041792E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q13)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>7.9769158902158552E-3</v>
       </c>
       <c r="S13" s="9">
-        <f t="shared" si="8"/>
-        <v>0.28491669995918356</v>
+        <f>Q13/MAX($Q$2:$Q$28)</f>
+        <v>0.4139704982018737</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>9</v>
+      <c r="B14" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D14" s="8">
-        <v>45511</v>
+        <v>45544</v>
       </c>
       <c r="E14" s="2">
-        <v>3.2899999999999999E-2</v>
+        <v>0.24390000000000001</v>
       </c>
       <c r="F14" s="1">
-        <v>455.4</v>
+        <v>144.28</v>
       </c>
       <c r="G14" s="1">
-        <f t="shared" si="0"/>
-        <v>14.982659999999999</v>
+        <f>E14*F14</f>
+        <v>35.189892</v>
       </c>
       <c r="H14" s="11">
-        <v>0.1</v>
+        <v>-2.8000000000000001E-2</v>
       </c>
       <c r="I14" s="11">
-        <v>0.18</v>
+        <v>0.18340000000000001</v>
       </c>
       <c r="J14" s="9">
-        <f t="shared" si="1"/>
-        <v>0.55555555555555558</v>
+        <f>IFERROR(H14/I14,"")</f>
+        <v>-0.15267175572519084</v>
       </c>
       <c r="K14" s="9">
-        <f t="shared" si="2"/>
-        <v>6.0770950849116732E-2</v>
+        <f>IFERROR(J14/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>-3.0773808280408366E-2</v>
       </c>
       <c r="L14" s="12">
-        <f t="shared" si="3"/>
-        <v>500.94</v>
+        <f>F14/(1-(F14*(1+H14)-F14)/(F14*(1+H14)))</f>
+        <v>140.24016</v>
       </c>
       <c r="M14" s="12">
-        <f t="shared" si="4"/>
-        <v>421.66666666666669</v>
+        <f>F14/(1+I14-H14)</f>
+        <v>119.10186561003798</v>
       </c>
       <c r="N14" s="12">
-        <f t="shared" si="5"/>
-        <v>45.54000000000002</v>
+        <f>L14-F14</f>
+        <v>-4.0398399999999981</v>
       </c>
       <c r="O14" s="12">
-        <f t="shared" si="6"/>
-        <v>-16.866666666666646</v>
+        <f>0.5*(M14-F14)</f>
+        <v>-12.589067194981013</v>
       </c>
       <c r="P14" s="15">
-        <f t="shared" si="7"/>
-        <v>28.673333333333375</v>
+        <f>N14+O14</f>
+        <v>-16.628907194981011</v>
       </c>
       <c r="Q14" s="12">
-        <f t="shared" si="9"/>
-        <v>9.6646862745097053</v>
+        <f>MAX($P$2:$P$280)-P14</f>
+        <v>100.05602854987877</v>
       </c>
       <c r="R14" s="9">
-        <f t="shared" si="10"/>
-        <v>0.10346947346210993</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q14)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>9.9944002824526607E-3</v>
       </c>
       <c r="S14" s="9">
-        <f t="shared" si="8"/>
-        <v>0.22189001699158839</v>
+        <f>Q14/MAX($Q$2:$Q$28)</f>
+        <v>0.33040580243567419</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C15" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D15" s="8">
-        <v>45482</v>
+        <v>45484</v>
       </c>
       <c r="E15" s="2">
-        <v>0.18820000000000001</v>
+        <v>0.24990000000000001</v>
       </c>
       <c r="F15" s="1">
-        <v>227.38</v>
+        <v>191.91</v>
       </c>
       <c r="G15" s="1">
-        <f t="shared" si="0"/>
-        <v>42.792915999999998</v>
+        <f>E15*F15</f>
+        <v>47.958309</v>
       </c>
       <c r="H15" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="I15" s="13">
-        <v>0.22500000000000001</v>
+        <f>227.4/F15-1</f>
+        <v>0.18493043614194149</v>
+      </c>
+      <c r="I15" s="11">
+        <v>0.37</v>
       </c>
       <c r="J15" s="9">
-        <f t="shared" si="1"/>
-        <v>0.44444444444444448</v>
+        <f>IFERROR(H15/I15,"")</f>
+        <v>0.49981198957281486</v>
       </c>
       <c r="K15" s="9">
-        <f t="shared" si="2"/>
-        <v>4.8616760679293387E-2</v>
+        <f>IFERROR(J15/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>0.10074632514902941</v>
       </c>
       <c r="L15" s="12">
-        <f t="shared" si="3"/>
-        <v>250.11800000000002</v>
+        <f>F15/(1-(F15*(1+H15)-F15)/(F15*(1+H15)))</f>
+        <v>227.39999999999998</v>
       </c>
       <c r="M15" s="12">
-        <f t="shared" si="4"/>
-        <v>202.11555555555555</v>
+        <f>F15/(1+I15-H15)</f>
+        <v>161.93986062322494</v>
       </c>
       <c r="N15" s="12">
-        <f t="shared" si="5"/>
-        <v>22.738000000000028</v>
+        <f>L15-F15</f>
+        <v>35.489999999999981</v>
       </c>
       <c r="O15" s="12">
-        <f t="shared" si="6"/>
-        <v>-12.632222222222225</v>
+        <f>0.5*(M15-F15)</f>
+        <v>-14.985069688387526</v>
       </c>
       <c r="P15" s="15">
-        <f t="shared" si="7"/>
-        <v>10.105777777777803</v>
+        <f>N15+O15</f>
+        <v>20.504930311612455</v>
       </c>
       <c r="Q15" s="12">
-        <f t="shared" si="9"/>
-        <v>28.232241830065277</v>
+        <f>MAX($P$2:$P$280)-P15</f>
+        <v>62.922191043285309</v>
       </c>
       <c r="R15" s="9">
-        <f t="shared" si="10"/>
-        <v>3.5420495687844132E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q15)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.5892644286847574E-2</v>
       </c>
       <c r="S15" s="9">
-        <f t="shared" si="8"/>
-        <v>0.6481796140559789</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+        <f>Q15/MAX($Q$2:$Q$28)</f>
+        <v>0.20778215289949825</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" t="s">
         <v>76</v>
-      </c>
-      <c r="C16" t="s">
-        <v>77</v>
       </c>
       <c r="D16" s="8">
         <v>45562</v>
@@ -1747,7 +1773,7 @@
         <v>56</v>
       </c>
       <c r="G16" s="1">
-        <f t="shared" si="0"/>
+        <f>E16*F16</f>
         <v>5.5999999999999999E-34</v>
       </c>
       <c r="H16" s="11">
@@ -1757,55 +1783,55 @@
         <v>0.19</v>
       </c>
       <c r="J16" s="9">
-        <f t="shared" si="1"/>
+        <f>IFERROR(H16/I16,"")</f>
         <v>0.42105263157894735</v>
       </c>
       <c r="K16" s="9">
-        <f t="shared" si="2"/>
-        <v>4.6057983801435831E-2</v>
+        <f>IFERROR(J16/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>8.4870923889126232E-2</v>
       </c>
       <c r="L16" s="12">
-        <f t="shared" si="3"/>
+        <f>F16/(1-(F16*(1+H16)-F16)/(F16*(1+H16)))</f>
         <v>60.480000000000004</v>
       </c>
       <c r="M16" s="12">
-        <f t="shared" si="4"/>
+        <f>F16/(1+I16-H16)</f>
         <v>50.450450450450454</v>
       </c>
       <c r="N16" s="12">
-        <f t="shared" si="5"/>
+        <f>L16-F16</f>
         <v>4.480000000000004</v>
       </c>
       <c r="O16" s="12">
-        <f t="shared" si="6"/>
+        <f>0.5*(M16-F16)</f>
         <v>-2.7747747747747731</v>
       </c>
       <c r="P16" s="15">
-        <f t="shared" si="7"/>
+        <f>N16+O16</f>
         <v>1.7052252252252309</v>
       </c>
       <c r="Q16" s="12">
-        <f t="shared" si="9"/>
-        <v>36.632794382617845</v>
+        <f>MAX($P$2:$P$280)-P16</f>
+        <v>81.72189612967253</v>
       </c>
       <c r="R16" s="9">
-        <f t="shared" si="10"/>
-        <v>2.7297944829305656E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q16)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.223662258659841E-2</v>
       </c>
       <c r="S16" s="9">
-        <f t="shared" si="8"/>
-        <v>0.8410465831102002</v>
-      </c>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+        <f>Q16/MAX($Q$2:$Q$28)</f>
+        <v>0.26986268652296996</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" t="s">
         <v>57</v>
-      </c>
-      <c r="C17" t="s">
-        <v>58</v>
       </c>
       <c r="D17" s="8">
         <v>45505</v>
@@ -1814,138 +1840,139 @@
         <v>1E-35</v>
       </c>
       <c r="F17" s="1">
-        <v>82.17</v>
+        <v>86.6</v>
       </c>
       <c r="G17" s="1">
-        <f t="shared" si="0"/>
-        <v>8.2170000000000005E-34</v>
+        <f>E17*F17</f>
+        <v>8.6599999999999988E-34</v>
       </c>
       <c r="H17" s="11">
-        <v>0.08</v>
+        <f>89.44/F17-1</f>
+        <v>3.2794457274826883E-2</v>
       </c>
       <c r="I17" s="11">
-        <v>0.19</v>
+        <v>0.17249999999999999</v>
       </c>
       <c r="J17" s="9">
-        <f t="shared" si="1"/>
-        <v>0.42105263157894735</v>
+        <f>IFERROR(H17/I17,"")</f>
+        <v>0.19011279579609788</v>
       </c>
       <c r="K17" s="9">
-        <f t="shared" si="2"/>
-        <v>4.6057983801435831E-2</v>
+        <f>IFERROR(J17/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>3.8320740478104097E-2</v>
       </c>
       <c r="L17" s="12">
-        <f t="shared" si="3"/>
-        <v>88.743600000000001</v>
+        <f>F17/(1-(F17*(1+H17)-F17)/(F17*(1+H17)))</f>
+        <v>89.44</v>
       </c>
       <c r="M17" s="12">
-        <f t="shared" si="4"/>
-        <v>74.027027027027032</v>
+        <f>F17/(1+I17-H17)</f>
+        <v>75.984538772119137</v>
       </c>
       <c r="N17" s="12">
-        <f t="shared" si="5"/>
-        <v>6.573599999999999</v>
+        <f>L17-F17</f>
+        <v>2.8400000000000034</v>
       </c>
       <c r="O17" s="12">
-        <f t="shared" si="6"/>
-        <v>-4.071486486486485</v>
+        <f>0.5*(M17-F17)</f>
+        <v>-5.3077306139404286</v>
       </c>
       <c r="P17" s="15">
-        <f t="shared" si="7"/>
-        <v>2.502113513513514</v>
+        <f>N17+O17</f>
+        <v>-2.4677306139404251</v>
       </c>
       <c r="Q17" s="12">
-        <f t="shared" si="9"/>
-        <v>35.835906094329566</v>
+        <f>MAX($P$2:$P$280)-P17</f>
+        <v>85.894851968838196</v>
       </c>
       <c r="R17" s="9">
-        <f t="shared" si="10"/>
-        <v>2.7904973223440644E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q17)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.1642141258509767E-2</v>
       </c>
       <c r="S17" s="9">
-        <f t="shared" si="8"/>
-        <v>0.82275094983185515</v>
+        <f>Q17/MAX($Q$2:$Q$28)</f>
+        <v>0.28364265403268213</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>37</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>12</v>
+        <v>38</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="C18" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D18" s="8">
-        <v>45574</v>
+        <v>45460</v>
       </c>
       <c r="E18" s="2">
-        <v>0.13370000000000001</v>
+        <v>0.1807</v>
       </c>
       <c r="F18" s="1">
-        <v>423.77</v>
+        <v>165.59</v>
       </c>
       <c r="G18" s="1">
-        <f t="shared" si="0"/>
-        <v>56.658049000000005</v>
+        <f>E18*F18</f>
+        <v>29.922113</v>
       </c>
       <c r="H18" s="11">
-        <v>7.0000000000000007E-2</v>
+        <v>6.7199999999999996E-2</v>
       </c>
       <c r="I18" s="11">
-        <v>0.19</v>
+        <v>0.16439999999999999</v>
       </c>
       <c r="J18" s="9">
-        <f t="shared" si="1"/>
-        <v>0.36842105263157898</v>
+        <f>IFERROR(H18/I18,"")</f>
+        <v>0.40875912408759124</v>
       </c>
       <c r="K18" s="9">
-        <f t="shared" si="2"/>
-        <v>4.0300735826256359E-2</v>
+        <f>IFERROR(J18/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>8.2392940709881665E-2</v>
       </c>
       <c r="L18" s="12">
-        <f t="shared" si="3"/>
-        <v>453.43389999999999</v>
+        <f>F18/(1-(F18*(1+H18)-F18)/(F18*(1+H18)))</f>
+        <v>176.717648</v>
       </c>
       <c r="M18" s="12">
-        <f t="shared" si="4"/>
-        <v>378.36607142857144</v>
+        <f>F18/(1+I18-H18)</f>
+        <v>150.92052497265766</v>
       </c>
       <c r="N18" s="12">
-        <f t="shared" si="5"/>
-        <v>29.663900000000012</v>
+        <f>L18-F18</f>
+        <v>11.127647999999994</v>
       </c>
       <c r="O18" s="12">
-        <f t="shared" si="6"/>
-        <v>-22.701964285714268</v>
+        <f>0.5*(M18-F18)</f>
+        <v>-7.3347375136711719</v>
       </c>
       <c r="P18" s="15">
-        <f t="shared" si="7"/>
-        <v>6.9619357142857439</v>
+        <f>N18+O18</f>
+        <v>3.7929104863288217</v>
       </c>
       <c r="Q18" s="12">
-        <f t="shared" si="9"/>
-        <v>31.376083893557336</v>
+        <f>MAX($P$2:$P$280)-P18</f>
+        <v>79.634210868568942</v>
       </c>
       <c r="R18" s="9">
-        <f t="shared" si="10"/>
-        <v>3.1871408917456927E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q18)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.2557417083600347E-2</v>
       </c>
       <c r="S18" s="9">
-        <f t="shared" si="8"/>
-        <v>0.7203585911146535</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+        <f>Q18/MAX($Q$2:$Q$28)</f>
+        <v>0.26296871587547221</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>77</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" t="s">
         <v>79</v>
-      </c>
-      <c r="C19" t="s">
-        <v>80</v>
       </c>
       <c r="D19" s="8">
         <v>45580</v>
@@ -1957,7 +1984,7 @@
         <v>20.399999999999999</v>
       </c>
       <c r="G19" s="1">
-        <f t="shared" si="0"/>
+        <f>E19*F19</f>
         <v>2.0399999999999999E-34</v>
       </c>
       <c r="H19" s="11">
@@ -1967,405 +1994,407 @@
         <v>0.15</v>
       </c>
       <c r="J19" s="9">
-        <f t="shared" si="1"/>
+        <f>IFERROR(H19/I19,"")</f>
         <v>0.33333333333333337</v>
       </c>
       <c r="K19" s="9">
-        <f t="shared" si="2"/>
-        <v>3.6462570509470042E-2</v>
+        <f>IFERROR(J19/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>6.7189481412224944E-2</v>
       </c>
       <c r="L19" s="12">
-        <f t="shared" si="3"/>
+        <f>F19/(1-(F19*(1+H19)-F19)/(F19*(1+H19)))</f>
         <v>21.419999999999998</v>
       </c>
       <c r="M19" s="12">
-        <f t="shared" si="4"/>
+        <f>F19/(1+I19-H19)</f>
         <v>18.545454545454547</v>
       </c>
       <c r="N19" s="12">
-        <f t="shared" si="5"/>
+        <f>L19-F19</f>
         <v>1.0199999999999996</v>
       </c>
       <c r="O19" s="12">
-        <f t="shared" si="6"/>
+        <f>0.5*(M19-F19)</f>
         <v>-0.92727272727272592</v>
       </c>
       <c r="P19" s="15">
-        <f t="shared" si="7"/>
+        <f>N19+O19</f>
         <v>9.2727272727273657E-2</v>
       </c>
       <c r="Q19" s="12">
-        <f t="shared" si="9"/>
-        <v>38.245292335115806</v>
+        <f>MAX($P$2:$P$280)-P19</f>
+        <v>83.33439408217049</v>
       </c>
       <c r="R19" s="9">
-        <f t="shared" si="10"/>
-        <v>2.6147008924333064E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q19)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.199984725411175E-2</v>
       </c>
       <c r="S19" s="9">
-        <f t="shared" si="8"/>
-        <v>0.87806767080161885</v>
+        <f>Q19/MAX($Q$2:$Q$28)</f>
+        <v>0.27518748991205688</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="D20" s="8">
-        <v>45580</v>
+        <v>45562</v>
       </c>
       <c r="E20" s="2">
-        <v>0.18010000000000001</v>
+        <v>4.0300000000000002E-2</v>
       </c>
       <c r="F20" s="1">
-        <v>133.19999999999999</v>
+        <v>668.82</v>
       </c>
       <c r="G20" s="1">
-        <f t="shared" si="0"/>
-        <v>23.989319999999999</v>
+        <f>E20*F20</f>
+        <v>26.953446000000003</v>
       </c>
       <c r="H20" s="11">
-        <v>0.05</v>
+        <f>553.57/F20-1</f>
+        <v>-0.17231841153075567</v>
       </c>
       <c r="I20" s="11">
-        <v>0.16</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="J20" s="9">
-        <f t="shared" si="1"/>
-        <v>0.3125</v>
+        <f>IFERROR(H20/I20,"")</f>
+        <v>-0.61542289832412733</v>
       </c>
       <c r="K20" s="9">
-        <f t="shared" si="2"/>
-        <v>3.4183659852628161E-2</v>
+        <f>IFERROR(J20/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>-0.12404983616281964</v>
       </c>
       <c r="L20" s="12">
-        <f t="shared" si="3"/>
-        <v>139.85999999999999</v>
+        <f>F20/(1-(F20*(1+H20)-F20)/(F20*(1+H20)))</f>
+        <v>553.57000000000005</v>
       </c>
       <c r="M20" s="12">
-        <f t="shared" si="4"/>
-        <v>120</v>
+        <f>F20/(1+I20-H20)</f>
+        <v>460.51884675555289</v>
       </c>
       <c r="N20" s="12">
-        <f t="shared" si="5"/>
-        <v>6.6599999999999966</v>
+        <f>L20-F20</f>
+        <v>-115.25</v>
       </c>
       <c r="O20" s="12">
-        <f t="shared" si="6"/>
-        <v>-6.5999999999999943</v>
+        <f>0.5*(M20-F20)</f>
+        <v>-104.15057662222358</v>
       </c>
       <c r="P20" s="15">
-        <f t="shared" si="7"/>
-        <v>6.0000000000002274E-2</v>
+        <f>N20+O20</f>
+        <v>-219.40057662222358</v>
       </c>
       <c r="Q20" s="12">
-        <f t="shared" si="9"/>
-        <v>38.278019607843078</v>
+        <f>MAX($P$2:$P$280)-P20</f>
+        <v>302.82769797712137</v>
       </c>
       <c r="R20" s="9">
-        <f t="shared" si="10"/>
-        <v>2.6124653528185725E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q20)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>3.3022078451871001E-3</v>
       </c>
       <c r="S20" s="9">
-        <f t="shared" si="8"/>
-        <v>0.87881905112533354</v>
+        <f>Q20/MAX($Q$2:$Q$28)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="5" t="s">
-        <v>16</v>
+      <c r="B21" s="6" t="s">
+        <v>42</v>
       </c>
       <c r="C21" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="D21" s="8">
-        <v>45460</v>
+        <v>45580</v>
       </c>
       <c r="E21" s="2">
-        <v>0.1807</v>
+        <v>0.19139999999999999</v>
       </c>
       <c r="F21" s="1">
-        <v>165.59</v>
+        <v>135.82</v>
       </c>
       <c r="G21" s="1">
-        <f t="shared" si="0"/>
-        <v>29.922113</v>
+        <f>E21*F21</f>
+        <v>25.995947999999999</v>
       </c>
       <c r="H21" s="11">
-        <v>0.06</v>
+        <v>0.1202</v>
       </c>
       <c r="I21" s="11">
-        <v>0.21</v>
+        <v>0.33710000000000001</v>
       </c>
       <c r="J21" s="9">
-        <f t="shared" si="1"/>
-        <v>0.2857142857142857</v>
+        <f>IFERROR(H21/I21,"")</f>
+        <v>0.35657075051913378</v>
       </c>
       <c r="K21" s="9">
-        <f t="shared" si="2"/>
-        <v>3.1253631865260027E-2</v>
+        <f>IFERROR(J21/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>7.1873411442445301E-2</v>
       </c>
       <c r="L21" s="12">
-        <f t="shared" si="3"/>
-        <v>175.52540000000002</v>
+        <f>F21/(1-(F21*(1+H21)-F21)/(F21*(1+H21)))</f>
+        <v>152.14556400000001</v>
       </c>
       <c r="M21" s="12">
-        <f t="shared" si="4"/>
-        <v>143.99130434782609</v>
+        <f>F21/(1+I21-H21)</f>
+        <v>111.61147177253677</v>
       </c>
       <c r="N21" s="12">
-        <f t="shared" si="5"/>
-        <v>9.9354000000000156</v>
+        <f>L21-F21</f>
+        <v>16.325564000000014</v>
       </c>
       <c r="O21" s="12">
-        <f t="shared" si="6"/>
-        <v>-10.799347826086958</v>
+        <f>0.5*(M21-F21)</f>
+        <v>-12.10426411373161</v>
       </c>
       <c r="P21" s="15">
-        <f t="shared" si="7"/>
-        <v>-0.86394782608694243</v>
+        <f>N21+O21</f>
+        <v>4.2212998862684046</v>
       </c>
       <c r="Q21" s="12">
-        <f t="shared" si="9"/>
-        <v>39.201967433930022</v>
+        <f>MAX($P$2:$P$280)-P21</f>
+        <v>79.205821468629352</v>
       </c>
       <c r="R21" s="9">
-        <f t="shared" si="10"/>
-        <v>2.5508923797903104E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q21)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.2625334621345541E-2</v>
       </c>
       <c r="S21" s="9">
-        <f t="shared" si="8"/>
-        <v>0.90003182441219065</v>
+        <f>Q21/MAX($Q$2:$Q$28)</f>
+        <v>0.26155408503819672</v>
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>7</v>
+      <c r="B22" s="6" t="s">
+        <v>60</v>
       </c>
       <c r="C22" t="s">
-        <v>6</v>
+        <v>61</v>
       </c>
       <c r="D22" s="8">
-        <v>45553</v>
+        <v>45580</v>
       </c>
       <c r="E22" s="2">
-        <v>1.0751999999999999</v>
+        <v>0.18010000000000001</v>
       </c>
       <c r="F22" s="1">
-        <v>51.15</v>
+        <v>133.19999999999999</v>
       </c>
       <c r="G22" s="1">
-        <f t="shared" si="0"/>
-        <v>54.996479999999998</v>
+        <f>E22*F22</f>
+        <v>23.989319999999999</v>
       </c>
       <c r="H22" s="11">
-        <v>7.1999999999999995E-2</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="I22" s="11">
-        <v>0.251</v>
+        <v>0.1623</v>
       </c>
       <c r="J22" s="9">
-        <f t="shared" si="1"/>
-        <v>0.28685258964143423</v>
+        <f>IFERROR(H22/I22,"")</f>
+        <v>3.0807147258163893E-2</v>
       </c>
       <c r="K22" s="9">
-        <f t="shared" si="2"/>
-        <v>3.1378148326874612E-2</v>
+        <f>IFERROR(J22/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>6.2097487441982379E-3</v>
       </c>
       <c r="L22" s="12">
-        <f t="shared" si="3"/>
-        <v>54.832799999999999</v>
+        <f>F22/(1-(F22*(1+H22)-F22)/(F22*(1+H22)))</f>
+        <v>133.86599999999999</v>
       </c>
       <c r="M22" s="12">
-        <f t="shared" si="4"/>
-        <v>43.384223918575067</v>
+        <f>F22/(1+I22-H22)</f>
+        <v>115.09548086062384</v>
       </c>
       <c r="N22" s="12">
-        <f t="shared" si="5"/>
-        <v>3.6828000000000003</v>
+        <f>L22-F22</f>
+        <v>0.66599999999999682</v>
       </c>
       <c r="O22" s="12">
-        <f t="shared" si="6"/>
-        <v>-3.8828880407124657</v>
+        <f>0.5*(M22-F22)</f>
+        <v>-9.0522595696880757</v>
       </c>
       <c r="P22" s="15">
-        <f t="shared" si="7"/>
-        <v>-0.20008804071246544</v>
+        <f>N22+O22</f>
+        <v>-8.3862595696880788</v>
       </c>
       <c r="Q22" s="12">
-        <f t="shared" si="9"/>
-        <v>38.538107648555545</v>
+        <f>MAX($P$2:$P$280)-P22</f>
+        <v>91.813380924585843</v>
       </c>
       <c r="R22" s="9">
-        <f t="shared" si="10"/>
-        <v>2.5948342070124485E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q22)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.0891658600627999E-2</v>
       </c>
       <c r="S22" s="9">
-        <f t="shared" si="8"/>
-        <v>0.88479037167664931</v>
+        <f>Q22/MAX($Q$2:$Q$28)</f>
+        <v>0.30318686678231904</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>39</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>20</v>
+        <v>36</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>23</v>
       </c>
       <c r="C23" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D23" s="8">
-        <v>45544</v>
+        <v>45482</v>
       </c>
       <c r="E23" s="2">
-        <v>0.24390000000000001</v>
+        <v>0.15210000000000001</v>
       </c>
       <c r="F23" s="1">
-        <v>144.28</v>
+        <v>147.01</v>
       </c>
       <c r="G23" s="1">
-        <f t="shared" si="0"/>
-        <v>35.189892</v>
+        <f>E23*F23</f>
+        <v>22.360220999999999</v>
       </c>
       <c r="H23" s="11">
-        <v>0.06</v>
+        <f>193.73/F23-1</f>
+        <v>0.3178015101013536</v>
       </c>
       <c r="I23" s="11">
-        <v>0.21</v>
+        <v>0.52380000000000004</v>
       </c>
       <c r="J23" s="9">
-        <f t="shared" si="1"/>
-        <v>0.2857142857142857</v>
+        <f>IFERROR(H23/I23,"")</f>
+        <v>0.60672300515722333</v>
       </c>
       <c r="K23" s="9">
-        <f t="shared" si="2"/>
-        <v>3.1253631865260027E-2</v>
+        <f>IFERROR(J23/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>0.12229621223214153</v>
       </c>
       <c r="L23" s="12">
-        <f t="shared" si="3"/>
-        <v>152.93680000000001</v>
+        <f>F23/(1-(F23*(1+H23)-F23)/(F23*(1+H23)))</f>
+        <v>193.72999999999996</v>
       </c>
       <c r="M23" s="12">
-        <f t="shared" si="4"/>
-        <v>125.46086956521741</v>
+        <f>F23/(1+I23-H23)</f>
+        <v>121.89899177432211</v>
       </c>
       <c r="N23" s="12">
-        <f t="shared" si="5"/>
-        <v>8.656800000000004</v>
+        <f>L23-F23</f>
+        <v>46.71999999999997</v>
       </c>
       <c r="O23" s="12">
-        <f t="shared" si="6"/>
-        <v>-9.4095652173912967</v>
+        <f>0.5*(M23-F23)</f>
+        <v>-12.555504112838939</v>
       </c>
       <c r="P23" s="15">
-        <f t="shared" si="7"/>
-        <v>-0.75276521739129265</v>
+        <f>N23+O23</f>
+        <v>34.164495887161031</v>
       </c>
       <c r="Q23" s="12">
-        <f t="shared" si="9"/>
-        <v>39.090784825234373</v>
+        <f>MAX($P$2:$P$280)-P23</f>
+        <v>49.262625467736733</v>
       </c>
       <c r="R23" s="9">
-        <f t="shared" si="10"/>
-        <v>2.5581476669521035E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q23)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>2.0299364690883635E-2</v>
       </c>
       <c r="S23" s="9">
-        <f t="shared" si="8"/>
-        <v>0.89747920032984307</v>
+        <f>Q23/MAX($Q$2:$Q$28)</f>
+        <v>0.16267542829407408</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>11</v>
+        <v>62</v>
       </c>
       <c r="C24" t="s">
-        <v>10</v>
+        <v>62</v>
       </c>
       <c r="D24" s="8">
-        <v>45544</v>
+        <v>45481</v>
       </c>
       <c r="E24" s="2">
-        <v>0.1928</v>
+        <v>2.8500000000000001E-2</v>
       </c>
       <c r="F24" s="1">
-        <v>188.12</v>
+        <v>700.32</v>
       </c>
       <c r="G24" s="1">
-        <f t="shared" si="0"/>
-        <v>36.269536000000002</v>
+        <f>E24*F24</f>
+        <v>19.959120000000002</v>
       </c>
       <c r="H24" s="11">
-        <v>0.1</v>
+        <v>-6.6500000000000004E-2</v>
       </c>
       <c r="I24" s="11">
-        <v>0.37</v>
+        <v>0.45340000000000003</v>
       </c>
       <c r="J24" s="9">
-        <f t="shared" si="1"/>
-        <v>0.27027027027027029</v>
+        <f>IFERROR(H24/I24,"")</f>
+        <v>-0.14666960741067489</v>
       </c>
       <c r="K24" s="9">
-        <f t="shared" si="2"/>
-        <v>2.956424635902976E-2</v>
+        <f>IFERROR(J24/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>-2.9563964582573606E-2</v>
       </c>
       <c r="L24" s="12">
-        <f t="shared" si="3"/>
-        <v>206.93200000000002</v>
+        <f>F24/(1-(F24*(1+H24)-F24)/(F24*(1+H24)))</f>
+        <v>653.74872000000005</v>
       </c>
       <c r="M24" s="12">
-        <f t="shared" si="4"/>
-        <v>148.1259842519685</v>
+        <f>F24/(1+I24-H24)</f>
+        <v>460.76715573392988</v>
       </c>
       <c r="N24" s="12">
-        <f t="shared" si="5"/>
-        <v>18.812000000000012</v>
+        <f>L24-F24</f>
+        <v>-46.571280000000002</v>
       </c>
       <c r="O24" s="12">
-        <f t="shared" si="6"/>
-        <v>-19.99700787401575</v>
+        <f>0.5*(M24-F24)</f>
+        <v>-119.77642213303508</v>
       </c>
       <c r="P24" s="15">
-        <f t="shared" si="7"/>
-        <v>-1.1850078740157386</v>
+        <f>N24+O24</f>
+        <v>-166.34770213303509</v>
       </c>
       <c r="Q24" s="12">
-        <f t="shared" si="9"/>
-        <v>39.523027481858819</v>
+        <f>MAX($P$2:$P$280)-P24</f>
+        <v>249.77482348793285</v>
       </c>
       <c r="R24" s="9">
-        <f t="shared" si="10"/>
-        <v>2.5301705454092625E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q24)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>4.0036060722041193E-3</v>
       </c>
       <c r="S24" s="9">
-        <f t="shared" si="8"/>
-        <v>0.90740299171827632</v>
-      </c>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+        <f>Q24/MAX($Q$2:$Q$28)</f>
+        <v>0.82480838165207504</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D25" s="8">
         <v>45483</v>
@@ -2374,68 +2403,69 @@
         <v>9.9999999999999997E-29</v>
       </c>
       <c r="F25" s="1">
-        <v>174.26</v>
+        <v>178.12</v>
       </c>
       <c r="G25" s="1">
-        <f t="shared" si="0"/>
-        <v>1.7425999999999999E-26</v>
+        <f>E25*F25</f>
+        <v>1.7812E-26</v>
       </c>
       <c r="H25" s="11">
-        <v>7.0000000000000007E-2</v>
+        <f>190.41/F25-1</f>
+        <v>6.8998428026049829E-2</v>
       </c>
       <c r="I25" s="11">
-        <v>0.26</v>
+        <v>0.26790000000000003</v>
       </c>
       <c r="J25" s="9">
-        <f t="shared" si="1"/>
-        <v>0.26923076923076927</v>
+        <f>IFERROR(H25/I25,"")</f>
+        <v>0.25755292282959996</v>
       </c>
       <c r="K25" s="9">
-        <f t="shared" si="2"/>
-        <v>2.945053771918734E-2</v>
+        <f>IFERROR(J25/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>5.1914541963370829E-2</v>
       </c>
       <c r="L25" s="12">
-        <f t="shared" si="3"/>
-        <v>186.45820000000001</v>
+        <f>F25/(1-(F25*(1+H25)-F25)/(F25*(1+H25)))</f>
+        <v>190.41</v>
       </c>
       <c r="M25" s="12">
-        <f t="shared" si="4"/>
-        <v>146.43697478991598</v>
+        <f>F25/(1+I25-H25)</f>
+        <v>148.56932726072878</v>
       </c>
       <c r="N25" s="12">
-        <f t="shared" si="5"/>
-        <v>12.198200000000014</v>
+        <f>L25-F25</f>
+        <v>12.289999999999992</v>
       </c>
       <c r="O25" s="12">
-        <f t="shared" si="6"/>
-        <v>-13.911512605042006</v>
+        <f>0.5*(M25-F25)</f>
+        <v>-14.77533636963561</v>
       </c>
       <c r="P25" s="15">
-        <f t="shared" si="7"/>
-        <v>-1.7133126050419918</v>
+        <f>N25+O25</f>
+        <v>-2.4853363696356183</v>
       </c>
       <c r="Q25" s="12">
-        <f t="shared" si="9"/>
-        <v>40.051332212885072</v>
+        <f>MAX($P$2:$P$280)-P25</f>
+        <v>85.912457724533382</v>
       </c>
       <c r="R25" s="9">
-        <f t="shared" si="10"/>
-        <v>2.4967958485992287E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q25)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.1639755473023065E-2</v>
       </c>
       <c r="S25" s="9">
-        <f t="shared" si="8"/>
-        <v>0.91953225721273213</v>
-      </c>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+        <f>Q25/MAX($Q$2:$Q$28)</f>
+        <v>0.28370079189725922</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" t="s">
         <v>30</v>
-      </c>
-      <c r="C26" t="s">
-        <v>31</v>
       </c>
       <c r="D26" s="8">
         <v>45481</v>
@@ -2444,278 +2474,280 @@
         <v>1E-22</v>
       </c>
       <c r="F26" s="1">
-        <v>246</v>
+        <v>169.34</v>
       </c>
       <c r="G26" s="1">
-        <f t="shared" si="0"/>
-        <v>2.4600000000000001E-20</v>
+        <f>E26*F26</f>
+        <v>1.6934000000000002E-20</v>
       </c>
       <c r="H26" s="11">
-        <v>0.1</v>
+        <f>174.52/F26-1</f>
+        <v>3.0589346876107371E-2</v>
       </c>
       <c r="I26" s="11">
-        <v>0.42</v>
+        <v>0.4259</v>
       </c>
       <c r="J26" s="9">
-        <f t="shared" si="1"/>
-        <v>0.23809523809523811</v>
+        <f>IFERROR(H26/I26,"")</f>
+        <v>7.1822838403633182E-2</v>
       </c>
       <c r="K26" s="9">
-        <f t="shared" si="2"/>
-        <v>2.6044693221050026E-2</v>
+        <f>IFERROR(J26/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>1.447721779768244E-2</v>
       </c>
       <c r="L26" s="12">
-        <f t="shared" si="3"/>
-        <v>270.60000000000002</v>
+        <f>F26/(1-(F26*(1+H26)-F26)/(F26*(1+H26)))</f>
+        <v>174.52000000000004</v>
       </c>
       <c r="M26" s="12">
-        <f t="shared" si="4"/>
-        <v>186.36363636363637</v>
+        <f>F26/(1+I26-H26)</f>
+        <v>121.36365448143965</v>
       </c>
       <c r="N26" s="12">
-        <f t="shared" si="5"/>
-        <v>24.600000000000023</v>
+        <f>L26-F26</f>
+        <v>5.1800000000000352</v>
       </c>
       <c r="O26" s="12">
-        <f t="shared" si="6"/>
-        <v>-29.818181818181813</v>
+        <f>0.5*(M26-F26)</f>
+        <v>-23.988172759280175</v>
       </c>
       <c r="P26" s="15">
-        <f t="shared" si="7"/>
-        <v>-5.2181818181817903</v>
+        <f>N26+O26</f>
+        <v>-18.80817275928014</v>
       </c>
       <c r="Q26" s="12">
-        <f t="shared" si="9"/>
-        <v>43.55620142602487</v>
+        <f>MAX($P$2:$P$280)-P26</f>
+        <v>102.2352941141779</v>
       </c>
       <c r="R26" s="9">
-        <f t="shared" si="10"/>
-        <v>2.2958843224618275E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q26)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>9.7813578829556158E-3</v>
       </c>
       <c r="S26" s="9">
-        <f t="shared" si="8"/>
-        <v>1</v>
+        <f>Q26/MAX($Q$2:$Q$28)</f>
+        <v>0.33760219027884886</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>34</v>
+      <c r="B27" s="7" t="s">
+        <v>26</v>
       </c>
       <c r="C27" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="D27" s="8">
-        <v>45562</v>
+        <v>45511</v>
       </c>
       <c r="E27" s="2">
-        <v>4.0300000000000002E-2</v>
+        <v>0.1933</v>
       </c>
       <c r="F27" s="1">
-        <v>668.82</v>
+        <v>77.53</v>
       </c>
       <c r="G27" s="1">
-        <f t="shared" si="0"/>
-        <v>26.953446000000003</v>
+        <f>E27*F27</f>
+        <v>14.986549</v>
       </c>
       <c r="H27" s="11">
-        <v>0.08</v>
+        <v>0.15</v>
       </c>
       <c r="I27" s="11">
-        <v>0.28000000000000003</v>
+        <v>0.26</v>
       </c>
       <c r="J27" s="9">
-        <f t="shared" si="1"/>
-        <v>0.2857142857142857</v>
+        <f>IFERROR(H27/I27,"")</f>
+        <v>0.57692307692307687</v>
       </c>
       <c r="K27" s="9">
-        <f t="shared" si="2"/>
-        <v>3.1253631865260027E-2</v>
+        <f>IFERROR(J27/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>0.11628948705962007</v>
       </c>
       <c r="L27" s="12">
-        <f t="shared" si="3"/>
-        <v>722.32560000000012</v>
+        <f>F27/(1-(F27*(1+H27)-F27)/(F27*(1+H27)))</f>
+        <v>89.159499999999994</v>
       </c>
       <c r="M27" s="12">
-        <f t="shared" si="4"/>
-        <v>557.35</v>
+        <f>F27/(1+I27-H27)</f>
+        <v>69.846846846846844</v>
       </c>
       <c r="N27" s="12">
-        <f t="shared" si="5"/>
-        <v>53.505600000000072</v>
+        <f>L27-F27</f>
+        <v>11.629499999999993</v>
       </c>
       <c r="O27" s="12">
-        <f t="shared" si="6"/>
-        <v>-55.735000000000014</v>
+        <f>0.5*(M27-F27)</f>
+        <v>-3.8415765765765784</v>
       </c>
       <c r="P27" s="15">
-        <f t="shared" si="7"/>
-        <v>-2.2293999999999414</v>
+        <f>N27+O27</f>
+        <v>7.7879234234234147</v>
       </c>
       <c r="Q27" s="12">
-        <f t="shared" si="9"/>
-        <v>40.567419607843021</v>
+        <f>MAX($P$2:$P$280)-P27</f>
+        <v>75.639197931474342</v>
       </c>
       <c r="R27" s="9">
-        <f t="shared" si="10"/>
-        <v>2.4650323083567953E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q27)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.3220658433025086E-2</v>
       </c>
       <c r="S27" s="9">
-        <f t="shared" si="8"/>
-        <v>0.93138102680377333</v>
+        <f>Q27/MAX($Q$2:$Q$28)</f>
+        <v>0.24977635281297447</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>41</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="C28" s="14" t="s">
-        <v>51</v>
+        <v>37</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28" t="s">
+        <v>28</v>
       </c>
       <c r="D28" s="8">
         <v>45511</v>
       </c>
       <c r="E28" s="2">
-        <v>1</v>
+        <v>3.2899999999999999E-2</v>
       </c>
       <c r="F28" s="1">
-        <v>10.4</v>
+        <v>455.4</v>
       </c>
       <c r="G28" s="1">
-        <f t="shared" si="0"/>
-        <v>10.4</v>
+        <f>E28*F28</f>
+        <v>14.982659999999999</v>
       </c>
       <c r="H28" s="11">
-        <v>0.2</v>
-      </c>
-      <c r="I28" s="13">
-        <v>1.7672000000000001</v>
+        <v>0.17460000000000001</v>
+      </c>
+      <c r="I28" s="11">
+        <v>0.15770000000000001</v>
       </c>
       <c r="J28" s="9">
-        <f t="shared" si="1"/>
-        <v>0.11317338162064282</v>
+        <f>IFERROR(H28/I28,"")</f>
+        <v>1.1071655041217501</v>
       </c>
       <c r="K28" s="9">
-        <f t="shared" si="2"/>
-        <v>1.2379777221413547E-2</v>
+        <f>IFERROR(J28/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>0.22316962817833491</v>
       </c>
       <c r="L28" s="12">
-        <f t="shared" si="3"/>
-        <v>12.48</v>
+        <f>F28/(1-(F28*(1+H28)-F28)/(F28*(1+H28)))</f>
+        <v>534.91283999999996</v>
       </c>
       <c r="M28" s="12">
-        <f t="shared" si="4"/>
-        <v>4.0511062636335309</v>
+        <f>F28/(1+I28-H28)</f>
+        <v>463.22856270979554</v>
       </c>
       <c r="N28" s="12">
-        <f t="shared" si="5"/>
-        <v>2.08</v>
+        <f>L28-F28</f>
+        <v>79.512839999999983</v>
       </c>
       <c r="O28" s="12">
-        <f t="shared" si="6"/>
-        <v>-3.1744468681832347</v>
+        <f>0.5*(M28-F28)</f>
+        <v>3.9142813548977813</v>
       </c>
       <c r="P28" s="15">
-        <f t="shared" si="7"/>
-        <v>-1.0944468681832347</v>
+        <f>N28+O28</f>
+        <v>83.427121354897764</v>
       </c>
       <c r="Q28" s="12">
-        <f t="shared" si="9"/>
-        <v>39.432466476026313</v>
+        <f>MAX($P$2:$P$280)-P28</f>
+        <v>0</v>
       </c>
       <c r="R28" s="9">
-        <f t="shared" si="10"/>
-        <v>2.5359813609629724E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q28)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>0</v>
       </c>
       <c r="S28" s="9">
-        <f t="shared" si="8"/>
-        <v>0.90532381578310406</v>
+        <f>Q28/MAX($Q$2:$Q$28)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>37</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C29" t="s">
-        <v>63</v>
+        <v>40</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>50</v>
       </c>
       <c r="D29" s="8">
-        <v>45481</v>
+        <v>45511</v>
       </c>
       <c r="E29" s="2">
-        <v>2.8500000000000001E-2</v>
+        <v>1</v>
       </c>
       <c r="F29" s="1">
-        <v>700.32</v>
+        <v>10.4</v>
       </c>
       <c r="G29" s="1">
-        <f t="shared" si="0"/>
-        <v>19.959120000000002</v>
+        <f>E29*F29</f>
+        <v>10.4</v>
       </c>
       <c r="H29" s="11">
-        <v>0.127</v>
-      </c>
-      <c r="I29" s="11">
-        <v>0.44</v>
+        <f>8.33/G29-1</f>
+        <v>-0.19903846153846161</v>
+      </c>
+      <c r="I29" s="13">
+        <v>2</v>
       </c>
       <c r="J29" s="9">
-        <f t="shared" si="1"/>
-        <v>0.28863636363636364</v>
+        <f>IFERROR(H29/I29,"")</f>
+        <v>-9.9519230769230804E-2</v>
       </c>
       <c r="K29" s="9">
-        <f t="shared" si="2"/>
-        <v>3.1573271282063824E-2</v>
+        <f>IFERROR(J29/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>-2.0059936517784469E-2</v>
       </c>
       <c r="L29" s="12">
-        <f t="shared" si="3"/>
-        <v>789.26064000000008</v>
+        <f>F29/(1-(F29*(1+H29)-F29)/(F29*(1+H29)))</f>
+        <v>8.33</v>
       </c>
       <c r="M29" s="12">
-        <f t="shared" si="4"/>
-        <v>533.37395277989344</v>
+        <f>F29/(1+I29-H29)</f>
+        <v>3.2509768560264503</v>
       </c>
       <c r="N29" s="12">
-        <f t="shared" si="5"/>
-        <v>88.94064000000003</v>
+        <f>L29-F29</f>
+        <v>-2.0700000000000003</v>
       </c>
       <c r="O29" s="12">
-        <f t="shared" si="6"/>
-        <v>-83.473023610053303</v>
+        <f>0.5*(M29-F29)</f>
+        <v>-3.574511571986775</v>
       </c>
       <c r="P29" s="15">
-        <f t="shared" si="7"/>
-        <v>5.4676163899467269</v>
+        <f>N29+O29</f>
+        <v>-5.6445115719867758</v>
       </c>
       <c r="Q29" s="12">
-        <f t="shared" si="9"/>
-        <v>32.870403217896353</v>
+        <f>MAX($P$2:$P$280)-P29</f>
+        <v>89.071632926884547</v>
       </c>
       <c r="R29" s="9">
-        <f t="shared" si="10"/>
-        <v>3.0422504809905958E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q29)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.1226918909422725E-2</v>
       </c>
       <c r="S29" s="9">
-        <f t="shared" si="8"/>
-        <v>0.7546664342096705</v>
-      </c>
-    </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+        <f>Q29/MAX($Q$2:$Q$28)</f>
+        <v>0.29413304503478377</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D30" s="8">
         <v>45511</v>
@@ -2727,7 +2759,7 @@
         <v>29.94</v>
       </c>
       <c r="G30" s="1">
-        <f t="shared" si="0"/>
+        <f>E30*F30</f>
         <v>2.9940000000000003E-21</v>
       </c>
       <c r="H30" s="13">
@@ -2737,68 +2769,68 @@
         <v>0.72</v>
       </c>
       <c r="J30" s="9">
-        <f t="shared" si="1"/>
+        <f>IFERROR(H30/I30,"")</f>
         <v>0.10416666666666667</v>
       </c>
       <c r="K30" s="9">
-        <f t="shared" si="2"/>
-        <v>1.1394553284209387E-2</v>
+        <f>IFERROR(J30/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>2.0996712941320293E-2</v>
       </c>
       <c r="L30" s="12">
-        <f t="shared" si="3"/>
+        <f>F30/(1-(F30*(1+H30)-F30)/(F30*(1+H30)))</f>
         <v>32.185499999999998</v>
       </c>
       <c r="M30" s="12">
-        <f t="shared" si="4"/>
+        <f>F30/(1+I30-H30)</f>
         <v>18.200607902735563</v>
       </c>
       <c r="N30" s="12">
-        <f t="shared" si="5"/>
+        <f>L30-F30</f>
         <v>2.2454999999999963</v>
       </c>
       <c r="O30" s="12">
-        <f t="shared" si="6"/>
+        <f>0.5*(M30-F30)</f>
         <v>-5.8696960486322194</v>
       </c>
       <c r="P30" s="15">
-        <f t="shared" si="7"/>
+        <f>N30+O30</f>
         <v>-3.6241960486322231</v>
       </c>
       <c r="Q30" s="12">
-        <f t="shared" si="9"/>
-        <v>41.962215656475301</v>
+        <f>MAX($P$2:$P$280)-P30</f>
+        <v>87.051317403529993</v>
       </c>
       <c r="R30" s="9">
-        <f t="shared" si="10"/>
-        <v>2.3830962792492281E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q30)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.1487476925414677E-2</v>
       </c>
       <c r="S30" s="9">
-        <f t="shared" si="8"/>
-        <v>0.96340393061463891</v>
+        <f>Q30/MAX($Q$2:$Q$28)</f>
+        <v>0.28746154326380913</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B31" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C31" t="s">
         <v>81</v>
-      </c>
-      <c r="C31" t="s">
-        <v>82</v>
       </c>
       <c r="D31" s="8">
         <v>45574</v>
       </c>
       <c r="E31" s="2">
-        <v>0.13370000000000001</v>
+        <v>0</v>
       </c>
       <c r="F31" s="1">
         <v>153.7552</v>
       </c>
       <c r="G31" s="1">
-        <f t="shared" si="0"/>
-        <v>20.557070240000002</v>
+        <f>E31*F31</f>
+        <v>0</v>
       </c>
       <c r="H31" s="11">
         <v>7.0000000000000007E-2</v>
@@ -2807,59 +2839,59 @@
         <v>0.19</v>
       </c>
       <c r="J31" s="9">
-        <f t="shared" si="1"/>
+        <f>IFERROR(H31/I31,"")</f>
         <v>0.36842105263157898</v>
       </c>
       <c r="K31" s="9">
-        <f t="shared" si="2"/>
-        <v>4.0300735826256359E-2</v>
+        <f>IFERROR(J31/SUBTOTAL(9,$J$2:$J$1048576),"")</f>
+        <v>7.4262058402985456E-2</v>
       </c>
       <c r="L31" s="12">
-        <f t="shared" si="3"/>
+        <f>F31/(1-(F31*(1+H31)-F31)/(F31*(1+H31)))</f>
         <v>164.51806400000001</v>
       </c>
       <c r="M31" s="12">
-        <f t="shared" si="4"/>
+        <f>F31/(1+I31-H31)</f>
         <v>137.28142857142859</v>
       </c>
       <c r="N31" s="12">
-        <f t="shared" si="5"/>
+        <f>L31-F31</f>
         <v>10.762864000000008</v>
       </c>
       <c r="O31" s="12">
-        <f t="shared" si="6"/>
+        <f>0.5*(M31-F31)</f>
         <v>-8.2368857142857053</v>
       </c>
       <c r="P31" s="15">
-        <f t="shared" si="7"/>
+        <f>N31+O31</f>
         <v>2.5259782857143023</v>
       </c>
       <c r="Q31" s="12">
-        <f t="shared" si="9"/>
-        <v>35.812041322128778</v>
+        <f>MAX($P$2:$P$280)-P31</f>
+        <v>80.901143069183462</v>
       </c>
       <c r="R31" s="9">
-        <f t="shared" si="10"/>
-        <v>2.7923568807625761E-2</v>
+        <f>IFERROR((SUBTOTAL(109,$Q$2:$Q$1048576)/Q31)/SUBTOTAL(109,$Q$2:$Q$1048576),0)</f>
+        <v>1.2360764781096351E-2</v>
       </c>
       <c r="S31" s="9">
-        <f t="shared" si="8"/>
-        <v>0.82220304226830598</v>
-      </c>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+        <f>Q31/MAX($Q$2:$Q$28)</f>
+        <v>0.26715238932766161</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B32" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C32" s="14" t="s">
         <v>83</v>
-      </c>
-      <c r="C32" s="14" t="s">
-        <v>84</v>
       </c>
       <c r="D32" s="8">
         <f ca="1">TODAY()-20</f>
-        <v>45594</v>
+        <v>45599</v>
       </c>
       <c r="E32" s="2">
         <v>1E-35</v>
@@ -2883,7 +2915,7 @@
       </c>
       <c r="K32" s="9">
         <f t="shared" si="2"/>
-        <v>2.1877542305682025E-2</v>
+        <v>4.0313688847334959E-2</v>
       </c>
       <c r="L32" s="12">
         <f t="shared" ref="L32" si="13">F32/(1-(F32*(1+H32)-F32)/(F32*(1+H32)))</f>
@@ -2907,21 +2939,41 @@
       </c>
       <c r="Q32" s="12">
         <f t="shared" si="9"/>
-        <v>155.8908767506997</v>
+        <v>200.97997849775439</v>
       </c>
       <c r="R32" s="9">
         <f t="shared" si="10"/>
-        <v>6.4147435747583708E-3</v>
+        <v>4.9756199969499615E-3</v>
       </c>
       <c r="S32" s="9">
         <f t="shared" si="8"/>
-        <v>3.5790741994676045</v>
+        <v>0.66367766172081932</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S32" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S30">
-      <sortCondition descending="1" ref="K1:K29"/>
+    <filterColumn colId="4">
+      <filters>
+        <filter val="0.0285"/>
+        <filter val="0.0329"/>
+        <filter val="0.0403"/>
+        <filter val="0.1337"/>
+        <filter val="0.1461"/>
+        <filter val="0.1521"/>
+        <filter val="0.1801"/>
+        <filter val="0.1807"/>
+        <filter val="0.1818"/>
+        <filter val="0.1882"/>
+        <filter val="0.1914"/>
+        <filter val="0.1928"/>
+        <filter val="0.1933"/>
+        <filter val="0.2439"/>
+        <filter val="1.0000"/>
+        <filter val="1.0752"/>
+      </filters>
+    </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A9:S31">
+      <sortCondition descending="1" ref="G1:G32"/>
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="R2:R32">

</xml_diff>